<commit_message>
Unify dashboard search, improve user creation flow, and regenerate SIM seed
</commit_message>
<xml_diff>
--- a/Libro1.xlsx
+++ b/Libro1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hug.leon\Desktop\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C337B92-00E4-463B-89C9-C9F9F0F2A971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942BB4D4-5500-4977-B97E-92BD10D20A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04497E22-FEAF-4EAE-A69F-4E82C41B14CF}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3374" uniqueCount="1363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3474" uniqueCount="1413">
   <si>
     <t>Bus</t>
   </si>
@@ -4166,13 +4166,163 @@
   </si>
   <si>
     <t>8956032256758023225</t>
+  </si>
+  <si>
+    <t>89560900000863707921</t>
+  </si>
+  <si>
+    <t>89560900000863707954</t>
+  </si>
+  <si>
+    <t>89560900000863707962</t>
+  </si>
+  <si>
+    <t>89560900000863707970</t>
+  </si>
+  <si>
+    <t>89560900000863707988</t>
+  </si>
+  <si>
+    <t>89560900000863707996</t>
+  </si>
+  <si>
+    <t>89560900000863708069</t>
+  </si>
+  <si>
+    <t>89560900000863708077</t>
+  </si>
+  <si>
+    <t>89560900000863708143</t>
+  </si>
+  <si>
+    <t>89560900000863708275</t>
+  </si>
+  <si>
+    <t>89560900000863708283</t>
+  </si>
+  <si>
+    <t>89560900000863708291</t>
+  </si>
+  <si>
+    <t>89560900000863708309</t>
+  </si>
+  <si>
+    <t>89560900000863708317</t>
+  </si>
+  <si>
+    <t>89560900000863708325</t>
+  </si>
+  <si>
+    <t>89560900000863708333</t>
+  </si>
+  <si>
+    <t>89560900000863708341</t>
+  </si>
+  <si>
+    <t>89560900000863708556</t>
+  </si>
+  <si>
+    <t>89560900000863708598</t>
+  </si>
+  <si>
+    <t>89560900000863708630</t>
+  </si>
+  <si>
+    <t>89560900000863708648</t>
+  </si>
+  <si>
+    <t>89560900000863708655</t>
+  </si>
+  <si>
+    <t>89560900000863708663</t>
+  </si>
+  <si>
+    <t>89560900000863708671</t>
+  </si>
+  <si>
+    <t>89560900000863708689</t>
+  </si>
+  <si>
+    <t>89560900000863708697</t>
+  </si>
+  <si>
+    <t>89560900000863708705</t>
+  </si>
+  <si>
+    <t>89560900000863708747</t>
+  </si>
+  <si>
+    <t>89560900000863708754</t>
+  </si>
+  <si>
+    <t>89560900000863708762</t>
+  </si>
+  <si>
+    <t>89560900000863708804</t>
+  </si>
+  <si>
+    <t>89560900000863708812</t>
+  </si>
+  <si>
+    <t>89560900000863708820</t>
+  </si>
+  <si>
+    <t>89560900000863708846</t>
+  </si>
+  <si>
+    <t>89560900000863708853</t>
+  </si>
+  <si>
+    <t>89560900000863708861</t>
+  </si>
+  <si>
+    <t>89560900000863708887</t>
+  </si>
+  <si>
+    <t>89560900000876934165</t>
+  </si>
+  <si>
+    <t>89560900000886139003</t>
+  </si>
+  <si>
+    <t>89560900000928036274</t>
+  </si>
+  <si>
+    <t>89560900000928036282</t>
+  </si>
+  <si>
+    <t>89560900000928036290</t>
+  </si>
+  <si>
+    <t>89560900000928036308</t>
+  </si>
+  <si>
+    <t>89560900000928036316</t>
+  </si>
+  <si>
+    <t>89560900000928036340</t>
+  </si>
+  <si>
+    <t>89560900000928036431</t>
+  </si>
+  <si>
+    <t>89560900000928036449</t>
+  </si>
+  <si>
+    <t>89560900000928036456</t>
+  </si>
+  <si>
+    <t>89560900000928036480</t>
+  </si>
+  <si>
+    <t>89560900000928036498</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4237,8 +4387,13 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4315,6 +4470,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFB34DBB"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9F6FC"/>
+        <bgColor rgb="FFF9F6FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFF9F6FC"/>
       </patternFill>
     </fill>
   </fills>
@@ -4438,7 +4605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4525,6 +4692,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22862,8 +23035,8 @@
       <c r="B655" s="29"/>
       <c r="C655" s="3"/>
       <c r="F655" s="10"/>
-      <c r="G655" t="s">
-        <v>1307</v>
+      <c r="G655" s="38" t="s">
+        <v>1339</v>
       </c>
       <c r="H655" s="31" t="s">
         <v>1308</v>
@@ -22879,8 +23052,8 @@
       <c r="B656" s="29"/>
       <c r="C656" s="3"/>
       <c r="F656" s="10"/>
-      <c r="G656" t="s">
-        <v>1309</v>
+      <c r="G656" s="38" t="s">
+        <v>1340</v>
       </c>
       <c r="H656" s="31" t="s">
         <v>1308</v>
@@ -22896,8 +23069,8 @@
       <c r="B657" s="29"/>
       <c r="C657" s="3"/>
       <c r="F657" s="10"/>
-      <c r="G657" t="s">
-        <v>1310</v>
+      <c r="G657" s="38" t="s">
+        <v>1338</v>
       </c>
       <c r="H657" s="31" t="s">
         <v>1308</v>
@@ -22913,15 +23086,15 @@
       <c r="B658" s="29"/>
       <c r="C658" s="3"/>
       <c r="F658" s="10"/>
-      <c r="G658" t="s">
-        <v>1311</v>
+      <c r="G658" s="38" t="s">
+        <v>166</v>
       </c>
       <c r="H658" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I658" t="e">
+      <c r="I658" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863574032</v>
       </c>
       <c r="J658" s="11"/>
     </row>
@@ -22930,8 +23103,8 @@
       <c r="B659" s="29"/>
       <c r="C659" s="3"/>
       <c r="F659" s="10"/>
-      <c r="G659" t="s">
-        <v>1312</v>
+      <c r="G659" s="38" t="s">
+        <v>1342</v>
       </c>
       <c r="H659" s="31" t="s">
         <v>1308</v>
@@ -22947,15 +23120,15 @@
       <c r="B660" s="29"/>
       <c r="C660" s="3"/>
       <c r="F660" s="10"/>
-      <c r="G660" t="s">
-        <v>698</v>
+      <c r="G660" s="38" t="s">
+        <v>269</v>
       </c>
       <c r="H660" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I660" t="str">
         <f t="shared" si="10"/>
-        <v>89560900000863586762</v>
+        <v>89560900000863574057</v>
       </c>
       <c r="J660" s="11"/>
     </row>
@@ -22964,15 +23137,15 @@
       <c r="B661" s="29"/>
       <c r="C661" s="3"/>
       <c r="F661" s="10"/>
-      <c r="G661" t="s">
-        <v>1313</v>
+      <c r="G661" s="38" t="s">
+        <v>1287</v>
       </c>
       <c r="H661" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I661" t="e">
+      <c r="I661" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863574065</v>
       </c>
       <c r="J661" s="11"/>
     </row>
@@ -22981,7 +23154,7 @@
       <c r="B662" s="29"/>
       <c r="C662" s="3"/>
       <c r="F662" s="10"/>
-      <c r="G662" t="s">
+      <c r="G662" s="38" t="s">
         <v>1314</v>
       </c>
       <c r="H662" s="31" t="s">
@@ -22998,8 +23171,8 @@
       <c r="B663" s="29"/>
       <c r="C663" s="3"/>
       <c r="F663" s="10"/>
-      <c r="G663" t="s">
-        <v>1315</v>
+      <c r="G663" s="38" t="s">
+        <v>1328</v>
       </c>
       <c r="H663" s="31" t="s">
         <v>1308</v>
@@ -23015,15 +23188,15 @@
       <c r="B664" s="29"/>
       <c r="C664" s="3"/>
       <c r="F664" s="10"/>
-      <c r="G664" t="s">
-        <v>885</v>
+      <c r="G664" s="38" t="s">
+        <v>1312</v>
       </c>
       <c r="H664" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I664" t="str">
+      <c r="I664" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585764</v>
+        <v>#N/A</v>
       </c>
       <c r="J664" s="11"/>
     </row>
@@ -23032,8 +23205,8 @@
       <c r="B665" s="29"/>
       <c r="C665" s="3"/>
       <c r="F665" s="10"/>
-      <c r="G665" t="s">
-        <v>1316</v>
+      <c r="G665" s="38" t="s">
+        <v>1311</v>
       </c>
       <c r="H665" s="31" t="s">
         <v>1308</v>
@@ -23049,8 +23222,8 @@
       <c r="B666" s="29"/>
       <c r="C666" s="3"/>
       <c r="F666" s="10"/>
-      <c r="G666" t="s">
-        <v>1317</v>
+      <c r="G666" s="38" t="s">
+        <v>1331</v>
       </c>
       <c r="H666" s="31" t="s">
         <v>1308</v>
@@ -23066,15 +23239,15 @@
       <c r="B667" s="29"/>
       <c r="C667" s="3"/>
       <c r="F667" s="10"/>
-      <c r="G667" t="s">
-        <v>1018</v>
+      <c r="G667" s="38" t="s">
+        <v>1326</v>
       </c>
       <c r="H667" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I667" t="str">
+      <c r="I667" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585756</v>
+        <v>#N/A</v>
       </c>
       <c r="J667" s="11"/>
     </row>
@@ -23083,15 +23256,15 @@
       <c r="B668" s="29"/>
       <c r="C668" s="3"/>
       <c r="F668" s="10"/>
-      <c r="G668" t="s">
-        <v>971</v>
+      <c r="G668" s="38" t="s">
+        <v>1105</v>
       </c>
       <c r="H668" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I668" t="str">
         <f t="shared" si="10"/>
-        <v>89560900000863585699</v>
+        <v>89560900000863574164</v>
       </c>
       <c r="J668" s="11"/>
     </row>
@@ -23100,15 +23273,15 @@
       <c r="B669" s="29"/>
       <c r="C669" s="3"/>
       <c r="F669" s="10"/>
-      <c r="G669" t="s">
-        <v>396</v>
+      <c r="G669" s="38" t="s">
+        <v>1316</v>
       </c>
       <c r="H669" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I669" t="str">
+      <c r="I669" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585681</v>
+        <v>#N/A</v>
       </c>
       <c r="J669" s="11"/>
     </row>
@@ -23117,15 +23290,15 @@
       <c r="B670" s="29"/>
       <c r="C670" s="3"/>
       <c r="F670" s="10"/>
-      <c r="G670" t="s">
-        <v>1105</v>
+      <c r="G670" s="38" t="s">
+        <v>1317</v>
       </c>
       <c r="H670" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I670" t="str">
+      <c r="I670" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863574164</v>
+        <v>#N/A</v>
       </c>
       <c r="J670" s="11"/>
     </row>
@@ -23134,15 +23307,15 @@
       <c r="B671" s="29"/>
       <c r="C671" s="3"/>
       <c r="F671" s="10"/>
-      <c r="G671" t="s">
-        <v>1287</v>
+      <c r="G671" s="38" t="s">
+        <v>1315</v>
       </c>
       <c r="H671" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I671" t="str">
+      <c r="I671" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863574065</v>
+        <v>#N/A</v>
       </c>
       <c r="J671" s="11"/>
     </row>
@@ -23151,15 +23324,15 @@
       <c r="B672" s="29"/>
       <c r="C672" s="3"/>
       <c r="F672" s="10"/>
-      <c r="G672" t="s">
-        <v>1318</v>
+      <c r="G672" s="38" t="s">
+        <v>1019</v>
       </c>
       <c r="H672" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I672" t="e">
+      <c r="I672" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863574206</v>
       </c>
       <c r="J672" s="11"/>
     </row>
@@ -23168,8 +23341,8 @@
       <c r="B673" s="29"/>
       <c r="C673" s="3"/>
       <c r="F673" s="10"/>
-      <c r="G673" t="s">
-        <v>1319</v>
+      <c r="G673" s="38" t="s">
+        <v>1337</v>
       </c>
       <c r="H673" s="31" t="s">
         <v>1308</v>
@@ -23185,8 +23358,8 @@
       <c r="B674" s="29"/>
       <c r="C674" s="3"/>
       <c r="F674" s="10"/>
-      <c r="G674" t="s">
-        <v>1320</v>
+      <c r="G674" s="38" t="s">
+        <v>1336</v>
       </c>
       <c r="H674" s="31" t="s">
         <v>1308</v>
@@ -23202,15 +23375,15 @@
       <c r="B675" s="29"/>
       <c r="C675" s="3"/>
       <c r="F675" s="10"/>
-      <c r="G675" t="s">
-        <v>445</v>
+      <c r="G675" s="38" t="s">
+        <v>1335</v>
       </c>
       <c r="H675" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I675" t="str">
+      <c r="I675" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585749</v>
+        <v>#N/A</v>
       </c>
       <c r="J675" s="11"/>
     </row>
@@ -23219,15 +23392,15 @@
       <c r="B676" s="29"/>
       <c r="C676" s="3"/>
       <c r="F676" s="10"/>
-      <c r="G676" t="s">
-        <v>1321</v>
+      <c r="G676" s="38" t="s">
+        <v>1297</v>
       </c>
       <c r="H676" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I676" t="e">
+      <c r="I676" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863574248</v>
       </c>
       <c r="J676" s="11"/>
     </row>
@@ -23236,8 +23409,8 @@
       <c r="B677" s="29"/>
       <c r="C677" s="3"/>
       <c r="F677" s="10"/>
-      <c r="G677" t="s">
-        <v>1322</v>
+      <c r="G677" s="38" t="s">
+        <v>1310</v>
       </c>
       <c r="H677" s="31" t="s">
         <v>1308</v>
@@ -23253,8 +23426,8 @@
       <c r="B678" s="29"/>
       <c r="C678" s="3"/>
       <c r="F678" s="10"/>
-      <c r="G678" t="s">
-        <v>1323</v>
+      <c r="G678" s="38" t="s">
+        <v>1313</v>
       </c>
       <c r="H678" s="31" t="s">
         <v>1308</v>
@@ -23270,15 +23443,15 @@
       <c r="B679" s="29"/>
       <c r="C679" s="3"/>
       <c r="F679" s="10"/>
-      <c r="G679" t="s">
-        <v>467</v>
+      <c r="G679" s="38" t="s">
+        <v>1307</v>
       </c>
       <c r="H679" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I679" t="str">
+      <c r="I679" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585632</v>
+        <v>#N/A</v>
       </c>
       <c r="J679" s="11"/>
     </row>
@@ -23287,8 +23460,8 @@
       <c r="B680" s="29"/>
       <c r="C680" s="3"/>
       <c r="F680" s="10"/>
-      <c r="G680" t="s">
-        <v>1324</v>
+      <c r="G680" s="38" t="s">
+        <v>1341</v>
       </c>
       <c r="H680" s="31" t="s">
         <v>1308</v>
@@ -23304,8 +23477,8 @@
       <c r="B681" s="29"/>
       <c r="C681" s="3"/>
       <c r="F681" s="10"/>
-      <c r="G681" t="s">
-        <v>1325</v>
+      <c r="G681" s="38" t="s">
+        <v>1309</v>
       </c>
       <c r="H681" s="31" t="s">
         <v>1308</v>
@@ -23321,15 +23494,15 @@
       <c r="B682" s="29"/>
       <c r="C682" s="3"/>
       <c r="F682" s="10"/>
-      <c r="G682" t="s">
-        <v>1326</v>
+      <c r="G682" s="38" t="s">
+        <v>1299</v>
       </c>
       <c r="H682" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I682" t="e">
+      <c r="I682" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585558</v>
       </c>
       <c r="J682" s="11"/>
     </row>
@@ -23338,15 +23511,15 @@
       <c r="B683" s="29"/>
       <c r="C683" s="3"/>
       <c r="F683" s="10"/>
-      <c r="G683" t="s">
-        <v>1327</v>
+      <c r="G683" s="38" t="s">
+        <v>1220</v>
       </c>
       <c r="H683" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I683" t="e">
+      <c r="I683" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585566</v>
       </c>
       <c r="J683" s="11"/>
     </row>
@@ -23355,8 +23528,8 @@
       <c r="B684" s="29"/>
       <c r="C684" s="3"/>
       <c r="F684" s="10"/>
-      <c r="G684" t="s">
-        <v>1328</v>
+      <c r="G684" s="38" t="s">
+        <v>1332</v>
       </c>
       <c r="H684" s="31" t="s">
         <v>1308</v>
@@ -23372,15 +23545,15 @@
       <c r="B685" s="29"/>
       <c r="C685" s="3"/>
       <c r="F685" s="10"/>
-      <c r="G685" t="s">
-        <v>1329</v>
+      <c r="G685" s="38" t="s">
+        <v>1241</v>
       </c>
       <c r="H685" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I685" t="e">
+      <c r="I685" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585582</v>
       </c>
       <c r="J685" s="11"/>
     </row>
@@ -23389,7 +23562,7 @@
       <c r="B686" s="29"/>
       <c r="C686" s="3"/>
       <c r="F686" s="10"/>
-      <c r="G686" t="s">
+      <c r="G686" s="38" t="s">
         <v>1330</v>
       </c>
       <c r="H686" s="31" t="s">
@@ -23406,15 +23579,15 @@
       <c r="B687" s="29"/>
       <c r="C687" s="3"/>
       <c r="F687" s="10"/>
-      <c r="G687" t="s">
-        <v>1241</v>
+      <c r="G687" s="38" t="s">
+        <v>1327</v>
       </c>
       <c r="H687" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I687" t="str">
+      <c r="I687" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585582</v>
+        <v>#N/A</v>
       </c>
       <c r="J687" s="11"/>
     </row>
@@ -23423,8 +23596,8 @@
       <c r="B688" s="29"/>
       <c r="C688" s="3"/>
       <c r="F688" s="10"/>
-      <c r="G688" t="s">
-        <v>1331</v>
+      <c r="G688" s="38" t="s">
+        <v>1325</v>
       </c>
       <c r="H688" s="31" t="s">
         <v>1308</v>
@@ -23440,15 +23613,15 @@
       <c r="B689" s="29"/>
       <c r="C689" s="3"/>
       <c r="F689" s="10"/>
-      <c r="G689" t="s">
-        <v>928</v>
+      <c r="G689" s="38" t="s">
+        <v>467</v>
       </c>
       <c r="H689" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I689" t="str">
         <f t="shared" si="10"/>
-        <v>89560900000863586739</v>
+        <v>89560900000863585632</v>
       </c>
       <c r="J689" s="11"/>
     </row>
@@ -23457,8 +23630,8 @@
       <c r="B690" s="29"/>
       <c r="C690" s="3"/>
       <c r="F690" s="10"/>
-      <c r="G690" t="s">
-        <v>1332</v>
+      <c r="G690" s="38" t="s">
+        <v>1323</v>
       </c>
       <c r="H690" s="31" t="s">
         <v>1308</v>
@@ -23474,15 +23647,15 @@
       <c r="B691" s="29"/>
       <c r="C691" s="3"/>
       <c r="F691" s="10"/>
-      <c r="G691" t="s">
-        <v>984</v>
+      <c r="G691" s="38" t="s">
+        <v>1321</v>
       </c>
       <c r="H691" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I691" t="str">
+      <c r="I691" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863586754</v>
+        <v>#N/A</v>
       </c>
       <c r="J691" s="11"/>
     </row>
@@ -23491,8 +23664,8 @@
       <c r="B692" s="29"/>
       <c r="C692" s="3"/>
       <c r="F692" s="10"/>
-      <c r="G692" t="s">
-        <v>1333</v>
+      <c r="G692" s="38" t="s">
+        <v>1320</v>
       </c>
       <c r="H692" s="31" t="s">
         <v>1308</v>
@@ -23508,15 +23681,15 @@
       <c r="B693" s="29"/>
       <c r="C693" s="3"/>
       <c r="F693" s="10"/>
-      <c r="G693" t="s">
-        <v>1220</v>
+      <c r="G693" s="38" t="s">
+        <v>1318</v>
       </c>
       <c r="H693" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I693" t="str">
+      <c r="I693" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863585566</v>
+        <v>#N/A</v>
       </c>
       <c r="J693" s="11"/>
     </row>
@@ -23525,15 +23698,15 @@
       <c r="B694" s="29"/>
       <c r="C694" s="3"/>
       <c r="F694" s="10"/>
-      <c r="G694" t="s">
-        <v>1299</v>
+      <c r="G694" s="38" t="s">
+        <v>396</v>
       </c>
       <c r="H694" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I694" t="str">
         <f t="shared" si="10"/>
-        <v>89560900000863585558</v>
+        <v>89560900000863585681</v>
       </c>
       <c r="J694" s="11"/>
     </row>
@@ -23542,15 +23715,15 @@
       <c r="B695" s="29"/>
       <c r="C695" s="3"/>
       <c r="F695" s="10"/>
-      <c r="G695" t="s">
-        <v>1334</v>
+      <c r="G695" s="38" t="s">
+        <v>971</v>
       </c>
       <c r="H695" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I695" t="e">
+      <c r="I695" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585699</v>
       </c>
       <c r="J695" s="11"/>
     </row>
@@ -23559,15 +23732,15 @@
       <c r="B696" s="29"/>
       <c r="C696" s="3"/>
       <c r="F696" s="10"/>
-      <c r="G696" t="s">
-        <v>1297</v>
+      <c r="G696" s="38" t="s">
+        <v>1319</v>
       </c>
       <c r="H696" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I696" t="str">
+      <c r="I696" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863574248</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="697" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
@@ -23575,8 +23748,8 @@
       <c r="B697" s="29"/>
       <c r="C697" s="3"/>
       <c r="F697" s="10"/>
-      <c r="G697" t="s">
-        <v>1335</v>
+      <c r="G697" s="38" t="s">
+        <v>1324</v>
       </c>
       <c r="H697" s="31" t="s">
         <v>1308</v>
@@ -23591,15 +23764,15 @@
       <c r="B698" s="29"/>
       <c r="C698" s="3"/>
       <c r="F698" s="10"/>
-      <c r="G698" t="s">
-        <v>269</v>
+      <c r="G698" s="38" t="s">
+        <v>1329</v>
       </c>
       <c r="H698" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I698" t="str">
+      <c r="I698" t="e">
         <f t="shared" si="10"/>
-        <v>89560900000863574057</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="699" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
@@ -23607,8 +23780,8 @@
       <c r="B699" s="29"/>
       <c r="C699" s="3"/>
       <c r="F699" s="10"/>
-      <c r="G699" t="s">
-        <v>1336</v>
+      <c r="G699" s="38" t="s">
+        <v>1322</v>
       </c>
       <c r="H699" s="31" t="s">
         <v>1308</v>
@@ -23623,15 +23796,15 @@
       <c r="B700" s="29"/>
       <c r="C700" s="3"/>
       <c r="F700" s="10"/>
-      <c r="G700" t="s">
-        <v>1337</v>
+      <c r="G700" s="38" t="s">
+        <v>445</v>
       </c>
       <c r="H700" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I700" t="e">
+      <c r="I700" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585749</v>
       </c>
     </row>
     <row r="701" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
@@ -23639,15 +23812,15 @@
       <c r="B701" s="29"/>
       <c r="C701" s="3"/>
       <c r="F701" s="10"/>
-      <c r="G701" t="s">
-        <v>1019</v>
+      <c r="G701" s="38" t="s">
+        <v>1018</v>
       </c>
       <c r="H701" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I701" t="str">
         <f t="shared" si="10"/>
-        <v>89560900000863574206</v>
+        <v>89560900000863585756</v>
       </c>
     </row>
     <row r="702" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
@@ -23655,15 +23828,15 @@
       <c r="B702" s="29"/>
       <c r="C702" s="3"/>
       <c r="F702" s="10"/>
-      <c r="G702" t="s">
-        <v>1338</v>
+      <c r="G702" s="38" t="s">
+        <v>885</v>
       </c>
       <c r="H702" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I702" t="e">
+      <c r="I702" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863585764</v>
       </c>
     </row>
     <row r="703" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
@@ -23671,8 +23844,8 @@
       <c r="B703" s="29"/>
       <c r="C703" s="3"/>
       <c r="F703" s="10"/>
-      <c r="G703" t="s">
-        <v>1339</v>
+      <c r="G703" s="38" t="s">
+        <v>1334</v>
       </c>
       <c r="H703" s="31" t="s">
         <v>1308</v>
@@ -23687,8 +23860,8 @@
       <c r="B704" s="29"/>
       <c r="C704" s="3"/>
       <c r="F704" s="10"/>
-      <c r="G704" t="s">
-        <v>1340</v>
+      <c r="G704" s="38" t="s">
+        <v>1333</v>
       </c>
       <c r="H704" s="31" t="s">
         <v>1308</v>
@@ -23703,15 +23876,15 @@
       <c r="B705" s="29"/>
       <c r="C705" s="3"/>
       <c r="F705" s="10"/>
-      <c r="G705" t="s">
-        <v>1341</v>
+      <c r="G705" s="38" t="s">
+        <v>928</v>
       </c>
       <c r="H705" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I705" t="e">
+      <c r="I705" t="str">
         <f t="shared" si="10"/>
-        <v>#N/A</v>
+        <v>89560900000863586739</v>
       </c>
     </row>
     <row r="706" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
@@ -23719,15 +23892,15 @@
       <c r="B706" s="29"/>
       <c r="C706" s="3"/>
       <c r="F706" s="10"/>
-      <c r="G706" t="s">
-        <v>1342</v>
+      <c r="G706" s="38" t="s">
+        <v>984</v>
       </c>
       <c r="H706" s="31" t="s">
         <v>1308</v>
       </c>
-      <c r="I706" t="e">
-        <f t="shared" ref="I706:I744" si="11">VLOOKUP(G706,D:D,1,0)</f>
-        <v>#N/A</v>
+      <c r="I706" t="str">
+        <f t="shared" ref="I706:I707" si="11">VLOOKUP(G706,D:D,1,0)</f>
+        <v>89560900000863586754</v>
       </c>
     </row>
     <row r="707" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
@@ -23735,15 +23908,15 @@
       <c r="B707" s="29"/>
       <c r="C707" s="3"/>
       <c r="F707" s="10"/>
-      <c r="G707" t="s">
-        <v>166</v>
+      <c r="G707" s="38" t="s">
+        <v>698</v>
       </c>
       <c r="H707" s="31" t="s">
         <v>1308</v>
       </c>
       <c r="I707" t="str">
         <f t="shared" si="11"/>
-        <v>89560900000863574032</v>
+        <v>89560900000863586762</v>
       </c>
     </row>
     <row r="708" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
@@ -23751,292 +23924,792 @@
       <c r="B708" s="29"/>
       <c r="C708" s="3"/>
       <c r="F708" s="10"/>
+      <c r="G708" s="39" t="s">
+        <v>1363</v>
+      </c>
+      <c r="H708" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I708" t="e">
+        <f t="shared" ref="I708:I757" si="12">VLOOKUP(G708,D:D,1,0)</f>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="709" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A709" s="30"/>
       <c r="B709" s="29"/>
       <c r="C709" s="3"/>
       <c r="F709" s="10"/>
+      <c r="G709" s="39" t="s">
+        <v>1364</v>
+      </c>
+      <c r="H709" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I709" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="710" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A710" s="30"/>
       <c r="B710" s="29"/>
       <c r="C710" s="3"/>
       <c r="F710" s="10"/>
+      <c r="G710" s="39" t="s">
+        <v>1365</v>
+      </c>
+      <c r="H710" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I710" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="711" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A711" s="30"/>
       <c r="B711" s="29"/>
       <c r="C711" s="3"/>
       <c r="F711" s="10"/>
+      <c r="G711" s="39" t="s">
+        <v>1366</v>
+      </c>
+      <c r="H711" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I711" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="712" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A712" s="30"/>
       <c r="B712" s="29"/>
       <c r="C712" s="3"/>
       <c r="F712" s="10"/>
+      <c r="G712" s="39" t="s">
+        <v>1367</v>
+      </c>
+      <c r="H712" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I712" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="713" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A713" s="30"/>
       <c r="B713" s="29"/>
       <c r="C713" s="3"/>
       <c r="F713" s="10"/>
+      <c r="G713" s="39" t="s">
+        <v>1368</v>
+      </c>
+      <c r="H713" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I713" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="714" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A714" s="30"/>
       <c r="B714" s="29"/>
       <c r="C714" s="3"/>
       <c r="F714" s="10"/>
+      <c r="G714" s="39" t="s">
+        <v>1369</v>
+      </c>
+      <c r="H714" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I714" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="715" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A715" s="30"/>
       <c r="B715" s="29"/>
       <c r="C715" s="3"/>
       <c r="F715" s="10"/>
+      <c r="G715" s="39" t="s">
+        <v>1370</v>
+      </c>
+      <c r="H715" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I715" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="716" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A716" s="30"/>
       <c r="B716" s="29"/>
       <c r="C716" s="3"/>
       <c r="F716" s="10"/>
+      <c r="G716" s="39" t="s">
+        <v>1371</v>
+      </c>
+      <c r="H716" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I716" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="717" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A717" s="30"/>
       <c r="B717" s="29"/>
       <c r="C717" s="3"/>
       <c r="F717" s="10"/>
+      <c r="G717" s="39" t="s">
+        <v>1372</v>
+      </c>
+      <c r="H717" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I717" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="718" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A718" s="30"/>
       <c r="B718" s="29"/>
       <c r="C718" s="3"/>
       <c r="F718" s="10"/>
+      <c r="G718" s="39" t="s">
+        <v>1373</v>
+      </c>
+      <c r="H718" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I718" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="719" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A719" s="30"/>
       <c r="B719" s="29"/>
       <c r="C719" s="3"/>
       <c r="F719" s="10"/>
+      <c r="G719" s="39" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H719" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I719" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="720" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A720" s="30"/>
       <c r="B720" s="29"/>
       <c r="C720" s="3"/>
       <c r="F720" s="10"/>
-    </row>
-    <row r="721" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G720" s="39" t="s">
+        <v>1375</v>
+      </c>
+      <c r="H720" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I720" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="721" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A721" s="33"/>
       <c r="B721" s="34"/>
       <c r="F721" s="10"/>
-    </row>
-    <row r="722" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G721" s="39" t="s">
+        <v>1376</v>
+      </c>
+      <c r="H721" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I721" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="722" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A722" s="33"/>
       <c r="B722" s="34"/>
       <c r="F722" s="10"/>
-    </row>
-    <row r="723" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G722" s="39" t="s">
+        <v>1377</v>
+      </c>
+      <c r="H722" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I722" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="723" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A723" s="33"/>
       <c r="B723" s="34"/>
       <c r="F723" s="10"/>
-    </row>
-    <row r="724" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G723" s="39" t="s">
+        <v>1378</v>
+      </c>
+      <c r="H723" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I723" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="724" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A724" s="33"/>
       <c r="B724" s="34"/>
       <c r="F724" s="10"/>
-    </row>
-    <row r="725" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G724" s="39" t="s">
+        <v>1379</v>
+      </c>
+      <c r="H724" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I724" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="725" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A725" s="33"/>
       <c r="B725" s="34"/>
       <c r="F725" s="10"/>
-    </row>
-    <row r="726" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G725" s="39" t="s">
+        <v>1380</v>
+      </c>
+      <c r="H725" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I725" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="726" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A726" s="33"/>
       <c r="B726" s="34"/>
       <c r="F726" s="10"/>
-    </row>
-    <row r="727" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G726" s="39" t="s">
+        <v>1381</v>
+      </c>
+      <c r="H726" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I726" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="727" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A727" s="33"/>
       <c r="B727" s="34"/>
       <c r="F727" s="10"/>
-    </row>
-    <row r="728" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G727" s="39" t="s">
+        <v>1382</v>
+      </c>
+      <c r="H727" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I727" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="728" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A728" s="33"/>
       <c r="B728" s="34"/>
       <c r="F728" s="10"/>
-    </row>
-    <row r="729" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G728" s="39" t="s">
+        <v>1383</v>
+      </c>
+      <c r="H728" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I728" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="729" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A729" s="33"/>
       <c r="B729" s="34"/>
       <c r="F729" s="10"/>
-    </row>
-    <row r="730" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G729" s="39" t="s">
+        <v>1384</v>
+      </c>
+      <c r="H729" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I729" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="730" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A730" s="33"/>
       <c r="B730" s="34"/>
       <c r="F730" s="10"/>
-    </row>
-    <row r="731" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G730" s="39" t="s">
+        <v>1385</v>
+      </c>
+      <c r="H730" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I730" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="731" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A731" s="33"/>
       <c r="B731" s="34"/>
       <c r="F731" s="10"/>
-    </row>
-    <row r="732" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G731" s="39" t="s">
+        <v>1386</v>
+      </c>
+      <c r="H731" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I731" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="732" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A732" s="33"/>
       <c r="B732" s="34"/>
       <c r="F732" s="10"/>
-    </row>
-    <row r="733" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G732" s="39" t="s">
+        <v>1387</v>
+      </c>
+      <c r="H732" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I732" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="733" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A733" s="33"/>
       <c r="B733" s="34"/>
       <c r="F733" s="10"/>
-    </row>
-    <row r="734" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G733" s="39" t="s">
+        <v>1388</v>
+      </c>
+      <c r="H733" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I733" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="734" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A734" s="33"/>
       <c r="B734" s="34"/>
       <c r="F734" s="10"/>
-    </row>
-    <row r="735" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G734" s="39" t="s">
+        <v>1389</v>
+      </c>
+      <c r="H734" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I734" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="735" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A735" s="33"/>
       <c r="B735" s="34"/>
       <c r="F735" s="10"/>
-    </row>
-    <row r="736" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G735" s="39" t="s">
+        <v>1390</v>
+      </c>
+      <c r="H735" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I735" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="736" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A736" s="33"/>
       <c r="B736" s="34"/>
       <c r="F736" s="10"/>
-    </row>
-    <row r="737" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G736" s="39" t="s">
+        <v>1391</v>
+      </c>
+      <c r="H736" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I736" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="737" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A737" s="33"/>
       <c r="B737" s="34"/>
       <c r="F737" s="10"/>
-    </row>
-    <row r="738" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G737" s="39" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H737" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I737" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="738" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A738" s="33"/>
       <c r="B738" s="34"/>
       <c r="F738" s="10"/>
-    </row>
-    <row r="739" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G738" s="39" t="s">
+        <v>1393</v>
+      </c>
+      <c r="H738" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I738" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="739" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A739" s="33"/>
       <c r="B739" s="34"/>
       <c r="F739" s="10"/>
-    </row>
-    <row r="740" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G739" s="39" t="s">
+        <v>1394</v>
+      </c>
+      <c r="H739" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I739" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="740" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A740" s="33"/>
       <c r="B740" s="34"/>
       <c r="F740" s="10"/>
-    </row>
-    <row r="741" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G740" s="39" t="s">
+        <v>1395</v>
+      </c>
+      <c r="H740" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I740" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="741" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A741" s="33"/>
       <c r="B741" s="34"/>
       <c r="F741" s="10"/>
-    </row>
-    <row r="742" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G741" s="39" t="s">
+        <v>1396</v>
+      </c>
+      <c r="H741" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I741" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="742" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A742" s="33"/>
       <c r="B742" s="34"/>
       <c r="F742" s="10"/>
-    </row>
-    <row r="743" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G742" s="39" t="s">
+        <v>1397</v>
+      </c>
+      <c r="H742" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I742" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="743" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A743" s="33"/>
       <c r="B743" s="34"/>
       <c r="F743" s="10"/>
-    </row>
-    <row r="744" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G743" s="39" t="s">
+        <v>1398</v>
+      </c>
+      <c r="H743" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I743" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="744" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A744" s="33"/>
       <c r="B744" s="34"/>
       <c r="F744" s="10"/>
-    </row>
-    <row r="745" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G744" s="39" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H744" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I744" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="745" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A745" s="33"/>
       <c r="B745" s="34"/>
-    </row>
-    <row r="746" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G745" s="39" t="s">
+        <v>1400</v>
+      </c>
+      <c r="H745" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I745" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="746" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A746" s="33"/>
       <c r="B746" s="34"/>
-    </row>
-    <row r="747" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G746" s="39" t="s">
+        <v>1401</v>
+      </c>
+      <c r="H746" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I746" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="747" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A747" s="33"/>
       <c r="B747" s="34"/>
-    </row>
-    <row r="748" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G747" s="39" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H747" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I747" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="748" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A748" s="33"/>
       <c r="B748" s="34"/>
-    </row>
-    <row r="749" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G748" s="39" t="s">
+        <v>1403</v>
+      </c>
+      <c r="H748" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I748" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="749" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A749" s="33"/>
       <c r="B749" s="34"/>
-    </row>
-    <row r="750" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G749" s="39" t="s">
+        <v>1404</v>
+      </c>
+      <c r="H749" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I749" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="750" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A750" s="33"/>
       <c r="B750" s="34"/>
-    </row>
-    <row r="751" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G750" s="39" t="s">
+        <v>1405</v>
+      </c>
+      <c r="H750" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I750" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="751" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A751" s="33"/>
       <c r="B751" s="34"/>
-    </row>
-    <row r="752" spans="1:6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G751" s="39" t="s">
+        <v>1406</v>
+      </c>
+      <c r="H751" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I751" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="752" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A752" s="33"/>
       <c r="B752" s="34"/>
-    </row>
-    <row r="753" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G752" s="39" t="s">
+        <v>1407</v>
+      </c>
+      <c r="H752" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I752" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="753" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A753" s="33"/>
       <c r="B753" s="34"/>
-    </row>
-    <row r="754" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G753" s="39" t="s">
+        <v>1408</v>
+      </c>
+      <c r="H753" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I753" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="754" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A754" s="33"/>
       <c r="B754" s="34"/>
-    </row>
-    <row r="755" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G754" s="39" t="s">
+        <v>1409</v>
+      </c>
+      <c r="H754" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I754" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="755" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A755" s="33"/>
       <c r="B755" s="34"/>
-    </row>
-    <row r="756" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G755" s="39" t="s">
+        <v>1410</v>
+      </c>
+      <c r="H755" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I755" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="756" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A756" s="33"/>
       <c r="B756" s="34"/>
-    </row>
-    <row r="757" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G756" s="39" t="s">
+        <v>1411</v>
+      </c>
+      <c r="H756" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I756" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="757" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A757" s="33"/>
       <c r="B757" s="34"/>
-    </row>
-    <row r="758" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G757" s="39" t="s">
+        <v>1412</v>
+      </c>
+      <c r="H757" s="31" t="s">
+        <v>1308</v>
+      </c>
+      <c r="I757" t="e">
+        <f t="shared" si="12"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="758" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A758" s="33"/>
       <c r="B758" s="34"/>
     </row>
-    <row r="759" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="759" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A759" s="33"/>
       <c r="B759" s="34"/>
     </row>
-    <row r="760" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="760" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A760" s="33"/>
       <c r="B760" s="34"/>
     </row>
-    <row r="761" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="761" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A761" s="33"/>
       <c r="B761" s="34"/>
     </row>
-    <row r="762" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="762" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A762" s="33"/>
       <c r="B762" s="34"/>
     </row>
-    <row r="763" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="763" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A763" s="33"/>
       <c r="B763" s="34"/>
     </row>
-    <row r="764" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="764" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A764" s="33"/>
       <c r="B764" s="34"/>
     </row>
-    <row r="765" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="765" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A765" s="33"/>
       <c r="B765" s="34"/>
     </row>
-    <row r="766" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="766" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A766" s="33"/>
       <c r="B766" s="34"/>
     </row>
-    <row r="767" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="767" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A767" s="33"/>
       <c r="B767" s="34"/>
     </row>
-    <row r="768" spans="1:2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="768" spans="1:9" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A768" s="33"/>
       <c r="B768" s="34"/>
     </row>

</xml_diff>